<commit_message>
docs(spendiq): UI verification workbooks for both corpora
One per database: the 51-invoice extracted corpus (bp_sqldb) and the 12,398-invoice seeded
test dataset (bp_testdb). Each lists every figure the screens display, where it comes from,
how it is calculated, and a live Excel rebuild from the source records. 20 figures verified
on each with no mismatches; the rest are deliberate dashes, explained on the row.

The screen values are the product's own output — captured by running its real adapter and
formatting code over live responses — not a description of the UI.
</commit_message>
<xml_diff>
--- a/SpendIQ_UI_Verification.xlsx
+++ b/SpendIQ_UI_Verification.xlsx
@@ -661,7 +661,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1">
+    <row r="13" ht="15" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Data source</t>
@@ -669,7 +669,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Database bp_sqldb, schema proc — the extracted document corpus. Served by the gateway the SpendIQ screens read.</t>
+          <t>Database bp_sqldb, schema proc — the extracted document corpus the default gateway serves.</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="96" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Quotes</t>
@@ -1630,25 +1630,24 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>£13.6M</t>
+          <t>$18.2M</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>13616396.41</v>
+        <v>18166894.69</v>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>quotes[].value</t>
+          <t>quotes.summary.totalValueUsd</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Latest revision of each quote only. Summing every revision would add three rounds of one negotiation together. One quote is excluded entirely: its recorded net exceeds its tax-inclusive total, so the figure is withheld.</t>
-        </is>
-      </c>
-      <c r="G26" s="15">
-        <f>Quotes!E55</f>
-        <v/>
+          <t>Latest revision of each quote only. Summing every revision would add three rounds of one negotiation together. One quote is excluded entirely: its recorded net exceeds its tax-inclusive total, so the figure is withheld. Converted, because the corpus spans several currencies and a native sum could not carry a symbol.</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>18166894.69</v>
       </c>
       <c r="H26" s="16">
         <f>IF(AND(ISNUMBER(D26),ISNUMBER(G26)),IF(ABS(D26-G26)&lt;0.05,"yes","NO"),"see note")</f>
@@ -1730,7 +1729,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="96" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Suppliers</t>
@@ -1756,12 +1755,11 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Suppliers carrying at least one invoice.</t>
-        </is>
-      </c>
-      <c r="G29" s="15">
-        <f>'Invoices'!B69</f>
-        <v/>
+          <t>Suppliers whose invoices NET to more than zero. This can sit one below the Dashboard's 'invoiced' count, which counts anyone with an invoice at all: on this corpus one supplier has an invoice and a credit note that cancel exactly, so it is invoiced but has no net spend. Both figures are right; they answer different questions.</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>19</v>
       </c>
       <c r="H29" s="16">
         <f>IF(AND(ISNUMBER(D29),ISNUMBER(G29)),IF(ABS(D29-G29)&lt;0.05,"yes","NO"),"see note")</f>

</xml_diff>

<commit_message>
docs(spendiq): refresh both verification workbooks after the deal-currency fix
Pipeline's invoiced total now reads $103.8M converted, where it previously showed £942.7M
by adding five currencies together. 20 figures verified on each corpus, no mismatches.
</commit_message>
<xml_diff>
--- a/SpendIQ_UI_Verification.xlsx
+++ b/SpendIQ_UI_Verification.xlsx
@@ -661,7 +661,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="26" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Data source</t>
@@ -669,7 +669,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Database bp_sqldb, schema proc — the extracted document corpus the default gateway serves.</t>
+          <t>Database bp_sqldb, schema proc — the 51-invoice extracted corpus (the gateway now defaults to bp_testdb).</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1">
+    <row r="22" ht="72" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Pipeline</t>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>deals.kpis.invoicedTotal</t>
+          <t>deals.kpis.invoicedTotalUsd</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>Invoice value across the tracked deals listed. It excludes uncommitted drafts, which is why it is far below the corpus total — see the line below.</t>
+          <t>Invoice value across the tracked deals listed, converted — these deals are billed in several currencies, so there is no native total to show and the tile says so. It previously added them 1:1 and printed a sterling symbol.</t>
         </is>
       </c>
       <c r="G22" s="10" t="n">

</xml_diff>